<commit_message>
Finalize : PCB is ordered
</commit_message>
<xml_diff>
--- a/QSTL_MicroDSUB_FFC/BOM.xlsx
+++ b/QSTL_MicroDSUB_FFC/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Jeonghyun\SNU_GIT\QSTL_MicroDSUB_FFC\QSTL_MicroDSUB_FFC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989A5E4B-DFC2-4502-B50D-FA1481F102E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD104C3B-8F22-4185-A343-809DC223789D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12800" yWindow="0" windowWidth="12800" windowHeight="15400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4380" yWindow="1920" windowWidth="19200" windowHeight="11260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RFSoC_FMC2_BOM" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <t>Footprint</t>
   </si>
   <si>
-    <t>J2, J3, J4, J5, J6</t>
+    <t>J1</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>

</xml_diff>